<commit_message>
data(orders): Ball acks 9684893-9684900 — all 5 geranium orders confirmed in full (24,700 plants)
</commit_message>
<xml_diff>
--- a/orders/Spring 2027/Orders-EHR-4.5-geranium.xlsx
+++ b/orders/Spring 2027/Orders-EHR-4.5-geranium.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G63"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -410,10 +410,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>ORDER DRAFT-EHR-SYNG-SYNG-2707</v>
+        <v>ORDER DRAFT-BALL-BALL-BALL-2707</v>
       </c>
       <c r="B1" t="str">
-        <v>EHR → Syngenta — Syngenta Mexico</v>
+        <v>Ball → Ball FloraPlant — Ball FloraPlant Mexico</v>
       </c>
       <c r="C1" t="str">
         <v>Ship wk 7 (2027-02-15)</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>1712025</v>
       </c>
       <c r="B3" t="str">
-        <v>Mojo Salmon</v>
+        <v>Fantasia Orange</v>
       </c>
       <c r="C3" t="str">
         <v>CALL</v>
@@ -459,10 +459,10 @@
         <v>400</v>
       </c>
       <c r="E3">
-        <v>0.5243</v>
+        <v>0.4581</v>
       </c>
       <c r="F3">
-        <v>209.72</v>
+        <v>183.24</v>
       </c>
       <c r="G3" t="str">
         <v/>
@@ -470,22 +470,22 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>1849107</v>
       </c>
       <c r="B4" t="str">
-        <v>Calliope Medium Pink Flame</v>
+        <v>Fantasia White Sizzle</v>
       </c>
       <c r="C4" t="str">
         <v>CALL</v>
       </c>
       <c r="D4">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E4">
-        <v>0.5983</v>
+        <v>0.4581</v>
       </c>
       <c r="F4">
-        <v>239.31</v>
+        <v>137.43</v>
       </c>
       <c r="G4" t="str">
         <v/>
@@ -493,22 +493,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>1712019</v>
       </c>
       <c r="B5" t="str">
-        <v>Calliope Medium Dark Red DL</v>
+        <v>Fantasia White</v>
       </c>
       <c r="C5" t="str">
         <v>CALL</v>
       </c>
       <c r="D5">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="E5">
-        <v>0.5983</v>
+        <v>0.4581</v>
       </c>
       <c r="F5">
-        <v>717.92</v>
+        <v>229.05</v>
       </c>
       <c r="G5" t="str">
         <v/>
@@ -516,22 +516,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>1741649</v>
       </c>
       <c r="B6" t="str">
-        <v>Calliope Medium Hot Rose</v>
+        <v>Solera Red</v>
       </c>
       <c r="C6" t="str">
         <v>CALL</v>
       </c>
       <c r="D6">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="E6">
-        <v>0.5983</v>
+        <v>0.5281</v>
       </c>
       <c r="F6">
-        <v>239.31</v>
+        <v>528.1</v>
       </c>
       <c r="G6" t="str">
         <v/>
@@ -539,131 +539,131 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>1712010</v>
       </c>
       <c r="B7" t="str">
-        <v>ORDER TOTAL</v>
+        <v>Fantasia Appleblossom</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>CALL</v>
       </c>
       <c r="D7">
-        <v>2400</v>
-      </c>
-      <c r="E7" t="str">
-        <v/>
+        <v>500</v>
+      </c>
+      <c r="E7">
+        <v>0.4581</v>
       </c>
       <c r="F7">
-        <v>1406.26</v>
+        <v>229.05</v>
       </c>
       <c r="G7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>1741629</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Fantasia Violet Imp</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D8">
+        <v>500</v>
+      </c>
+      <c r="E8">
+        <v>0.4581</v>
+      </c>
+      <c r="F8">
+        <v>229.05</v>
+      </c>
+      <c r="G8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ORDER DRAFT-EHR-DUMM-DUMM-2707</v>
+        <v>1711998</v>
       </c>
       <c r="B9" t="str">
-        <v>EHR → Dummen — Dummen Oglevee Mexico</v>
+        <v>Fantasia Shocking Pink</v>
       </c>
       <c r="C9" t="str">
-        <v>Ship wk 7 (2027-02-15)</v>
-      </c>
-      <c r="D9" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D9">
+        <v>500</v>
+      </c>
+      <c r="E9">
+        <v>0.4581</v>
+      </c>
+      <c r="F9">
+        <v>229.05</v>
+      </c>
+      <c r="G9" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Material #</v>
+        <v/>
       </c>
       <c r="B10" t="str">
-        <v>Variety</v>
+        <v>ORDER TOTAL</v>
       </c>
       <c r="C10" t="str">
-        <v>Form</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Qty</v>
+        <v/>
+      </c>
+      <c r="D10">
+        <v>3700</v>
       </c>
       <c r="E10" t="str">
-        <v>$/unit</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Ext $</v>
+        <v/>
+      </c>
+      <c r="F10">
+        <v>1764.97</v>
       </c>
       <c r="G10" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-      <c r="B11" t="str">
-        <v>Brocade Fire</v>
-      </c>
-      <c r="C11" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D11">
-        <v>300</v>
-      </c>
-      <c r="E11">
-        <v>0.6126</v>
-      </c>
-      <c r="F11">
-        <v>183.78</v>
-      </c>
-      <c r="G11" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>ORDER DRAFT-EHR-DUMM-DUMM-2707</v>
       </c>
       <c r="B12" t="str">
-        <v>Brocade Vancouver Centennial</v>
+        <v>EHR → Dummen — Dummen Oglevee Mexico</v>
       </c>
       <c r="C12" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D12">
-        <v>300</v>
-      </c>
-      <c r="E12">
-        <v>0.5686</v>
-      </c>
-      <c r="F12">
-        <v>170.58</v>
-      </c>
-      <c r="G12" t="str">
+        <v>Ship wk 7 (2027-02-15)</v>
+      </c>
+      <c r="D12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>Material #</v>
       </c>
       <c r="B13" t="str">
-        <v>Big Eeze Pink Batik</v>
+        <v>Variety</v>
       </c>
       <c r="C13" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D13">
-        <v>400</v>
-      </c>
-      <c r="E13">
-        <v>0.5325</v>
-      </c>
-      <c r="F13">
-        <v>213</v>
+        <v>Form</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Qty</v>
+      </c>
+      <c r="E13" t="str">
+        <v>$/unit</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Ext $</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>Notes</v>
       </c>
     </row>
     <row r="14">
@@ -671,7 +671,7 @@
         <v/>
       </c>
       <c r="B14" t="str">
-        <v>Brocade Fire Night</v>
+        <v>Brocade Fire</v>
       </c>
       <c r="C14" t="str">
         <v>CALL</v>
@@ -694,7 +694,7 @@
         <v/>
       </c>
       <c r="B15" t="str">
-        <v>Brocade Wilhelm Langguth</v>
+        <v>Brocade Vancouver Centennial</v>
       </c>
       <c r="C15" t="str">
         <v>CALL</v>
@@ -717,128 +717,128 @@
         <v/>
       </c>
       <c r="B16" t="str">
-        <v>ORDER TOTAL</v>
+        <v>Big Eeze Pink Batik</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>CALL</v>
       </c>
       <c r="D16">
-        <v>1600</v>
-      </c>
-      <c r="E16" t="str">
-        <v/>
+        <v>400</v>
+      </c>
+      <c r="E16">
+        <v>0.5325</v>
       </c>
       <c r="F16">
-        <v>921.72</v>
+        <v>213</v>
       </c>
       <c r="G16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v>Brocade Fire Night</v>
+      </c>
+      <c r="C17" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D17">
+        <v>300</v>
+      </c>
+      <c r="E17">
+        <v>0.6126</v>
+      </c>
+      <c r="F17">
+        <v>183.78</v>
+      </c>
+      <c r="G17" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ORDER DRAFT-EHR-SYNG-SYNG-2708</v>
+        <v/>
       </c>
       <c r="B18" t="str">
-        <v>EHR → Syngenta — Syngenta Mexico</v>
+        <v>Brocade Wilhelm Langguth</v>
       </c>
       <c r="C18" t="str">
-        <v>Ship wk 8 (2027-02-22)</v>
-      </c>
-      <c r="D18" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D18">
+        <v>300</v>
+      </c>
+      <c r="E18">
+        <v>0.5686</v>
+      </c>
+      <c r="F18">
+        <v>170.58</v>
+      </c>
+      <c r="G18" t="str">
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Material #</v>
+        <v/>
       </c>
       <c r="B19" t="str">
-        <v>Variety</v>
+        <v>ORDER TOTAL</v>
       </c>
       <c r="C19" t="str">
-        <v>Form</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Qty</v>
+        <v/>
+      </c>
+      <c r="D19">
+        <v>1600</v>
       </c>
       <c r="E19" t="str">
-        <v>$/unit</v>
-      </c>
-      <c r="F19" t="str">
-        <v>Ext $</v>
+        <v/>
+      </c>
+      <c r="F19">
+        <v>921.72</v>
       </c>
       <c r="G19" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v/>
-      </c>
-      <c r="B20" t="str">
-        <v>Mojo Salmon</v>
-      </c>
-      <c r="C20" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D20">
-        <v>500</v>
-      </c>
-      <c r="E20">
-        <v>0.5243</v>
-      </c>
-      <c r="F20">
-        <v>262.15</v>
-      </c>
-      <c r="G20" t="str">
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v>ORDER DRAFT-EHR-SYNG-SYNG-2707</v>
       </c>
       <c r="B21" t="str">
-        <v>Calliope Medium Pink Flame</v>
+        <v>EHR → Syngenta — Syngenta Mexico</v>
       </c>
       <c r="C21" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D21">
-        <v>400</v>
-      </c>
-      <c r="E21">
-        <v>0.5983</v>
-      </c>
-      <c r="F21">
-        <v>239.31</v>
-      </c>
-      <c r="G21" t="str">
+        <v>Ship wk 7 (2027-02-15)</v>
+      </c>
+      <c r="D21" t="str">
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>Material #</v>
       </c>
       <c r="B22" t="str">
-        <v>Calliope Medium Hot Rose</v>
+        <v>Variety</v>
       </c>
       <c r="C22" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D22">
-        <v>400</v>
-      </c>
-      <c r="E22">
-        <v>0.5983</v>
-      </c>
-      <c r="F22">
-        <v>239.31</v>
+        <v>Form</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Qty</v>
+      </c>
+      <c r="E22" t="str">
+        <v>$/unit</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Ext $</v>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>Notes</v>
       </c>
     </row>
     <row r="23">
@@ -846,19 +846,19 @@
         <v/>
       </c>
       <c r="B23" t="str">
-        <v>Calliope Medium Dark Red DL</v>
+        <v>Mojo Salmon</v>
       </c>
       <c r="C23" t="str">
         <v>CALL</v>
       </c>
       <c r="D23">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="E23">
-        <v>0.5983</v>
+        <v>0.5243</v>
       </c>
       <c r="F23">
-        <v>598.27</v>
+        <v>209.72</v>
       </c>
       <c r="G23" t="str">
         <v/>
@@ -869,128 +869,128 @@
         <v/>
       </c>
       <c r="B24" t="str">
-        <v>ORDER TOTAL</v>
+        <v>Calliope Medium Pink Flame</v>
       </c>
       <c r="C24" t="str">
-        <v/>
+        <v>CALL</v>
       </c>
       <c r="D24">
-        <v>2300</v>
-      </c>
-      <c r="E24" t="str">
-        <v/>
+        <v>400</v>
+      </c>
+      <c r="E24">
+        <v>0.5983</v>
       </c>
       <c r="F24">
-        <v>1339.04</v>
+        <v>239.31</v>
       </c>
       <c r="G24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+      <c r="B25" t="str">
+        <v>Calliope Medium Dark Red DL</v>
+      </c>
+      <c r="C25" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D25">
+        <v>1200</v>
+      </c>
+      <c r="E25">
+        <v>0.5983</v>
+      </c>
+      <c r="F25">
+        <v>717.92</v>
+      </c>
+      <c r="G25" t="str">
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ORDER DRAFT-EHR-SYNG-SYNG-2709</v>
+        <v/>
       </c>
       <c r="B26" t="str">
-        <v>EHR → Syngenta — Syngenta Mexico</v>
+        <v>Calliope Medium Hot Rose</v>
       </c>
       <c r="C26" t="str">
-        <v>Ship wk 9 (2027-03-01)</v>
-      </c>
-      <c r="D26" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D26">
+        <v>400</v>
+      </c>
+      <c r="E26">
+        <v>0.5983</v>
+      </c>
+      <c r="F26">
+        <v>239.31</v>
+      </c>
+      <c r="G26" t="str">
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Material #</v>
+        <v/>
       </c>
       <c r="B27" t="str">
-        <v>Variety</v>
+        <v>ORDER TOTAL</v>
       </c>
       <c r="C27" t="str">
-        <v>Form</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Qty</v>
+        <v/>
+      </c>
+      <c r="D27">
+        <v>2400</v>
       </c>
       <c r="E27" t="str">
-        <v>$/unit</v>
-      </c>
-      <c r="F27" t="str">
-        <v>Ext $</v>
+        <v/>
+      </c>
+      <c r="F27">
+        <v>1406.26</v>
       </c>
       <c r="G27" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v/>
-      </c>
-      <c r="B28" t="str">
-        <v>Mojo Salmon</v>
-      </c>
-      <c r="C28" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D28">
-        <v>300</v>
-      </c>
-      <c r="E28">
-        <v>0.5243</v>
-      </c>
-      <c r="F28">
-        <v>157.29</v>
-      </c>
-      <c r="G28" t="str">
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>ORDER DRAFT-EHR-SYNG-SYNG-2708</v>
       </c>
       <c r="B29" t="str">
-        <v>Caldera Lavender Glow</v>
+        <v>EHR → Syngenta — Syngenta Mexico</v>
       </c>
       <c r="C29" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D29">
-        <v>300</v>
-      </c>
-      <c r="E29">
-        <v>0.5243</v>
-      </c>
-      <c r="F29">
-        <v>157.29</v>
-      </c>
-      <c r="G29" t="str">
+        <v>Ship wk 8 (2027-02-22)</v>
+      </c>
+      <c r="D29" t="str">
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v/>
+        <v>Material #</v>
       </c>
       <c r="B30" t="str">
-        <v>Caldera Hot Pink</v>
+        <v>Variety</v>
       </c>
       <c r="C30" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D30">
-        <v>300</v>
-      </c>
-      <c r="E30">
-        <v>0.5243</v>
-      </c>
-      <c r="F30">
-        <v>157.29</v>
+        <v>Form</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Qty</v>
+      </c>
+      <c r="E30" t="str">
+        <v>$/unit</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Ext $</v>
       </c>
       <c r="G30" t="str">
-        <v/>
+        <v>Notes</v>
       </c>
     </row>
     <row r="31">
@@ -998,19 +998,19 @@
         <v/>
       </c>
       <c r="B31" t="str">
-        <v>Calliope Medium Pink Flame</v>
+        <v>Mojo Salmon</v>
       </c>
       <c r="C31" t="str">
         <v>CALL</v>
       </c>
       <c r="D31">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="E31">
-        <v>0.5983</v>
+        <v>0.5243</v>
       </c>
       <c r="F31">
-        <v>179.48</v>
+        <v>262.15</v>
       </c>
       <c r="G31" t="str">
         <v/>
@@ -1021,19 +1021,19 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>Calliope Medium Hot Rose</v>
+        <v>Calliope Medium Pink Flame</v>
       </c>
       <c r="C32" t="str">
         <v>CALL</v>
       </c>
       <c r="D32">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E32">
         <v>0.5983</v>
       </c>
       <c r="F32">
-        <v>179.48</v>
+        <v>239.31</v>
       </c>
       <c r="G32" t="str">
         <v/>
@@ -1044,19 +1044,19 @@
         <v/>
       </c>
       <c r="B33" t="str">
-        <v>Calliope Medium Dark Red DL</v>
+        <v>Calliope Medium Hot Rose</v>
       </c>
       <c r="C33" t="str">
         <v>CALL</v>
       </c>
       <c r="D33">
-        <v>1200</v>
+        <v>400</v>
       </c>
       <c r="E33">
         <v>0.5983</v>
       </c>
       <c r="F33">
-        <v>717.92</v>
+        <v>239.31</v>
       </c>
       <c r="G33" t="str">
         <v/>
@@ -1067,82 +1067,82 @@
         <v/>
       </c>
       <c r="B34" t="str">
+        <v>Calliope Medium Dark Red DL</v>
+      </c>
+      <c r="C34" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D34">
+        <v>1000</v>
+      </c>
+      <c r="E34">
+        <v>0.5983</v>
+      </c>
+      <c r="F34">
+        <v>598.27</v>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
         <v>ORDER TOTAL</v>
       </c>
-      <c r="C34" t="str">
-        <v/>
-      </c>
-      <c r="D34">
-        <v>2700</v>
-      </c>
-      <c r="E34" t="str">
-        <v/>
-      </c>
-      <c r="F34">
-        <v>1548.75</v>
-      </c>
-      <c r="G34" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>ORDER DRAFT-EHR-SYNG-SYNG-2710</v>
-      </c>
-      <c r="B36" t="str">
-        <v>EHR → Syngenta — Syngenta Mexico</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Ship wk 10 (2027-03-08)</v>
-      </c>
-      <c r="D36" t="str">
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35">
+        <v>2300</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35">
+        <v>1339.04</v>
+      </c>
+      <c r="G35" t="str">
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Material #</v>
+        <v>ORDER DRAFT-EHR-SYNG-SYNG-2709</v>
       </c>
       <c r="B37" t="str">
-        <v>Variety</v>
+        <v>EHR → Syngenta — Syngenta Mexico</v>
       </c>
       <c r="C37" t="str">
-        <v>Form</v>
+        <v>Ship wk 9 (2027-03-01)</v>
       </c>
       <c r="D37" t="str">
-        <v>Qty</v>
-      </c>
-      <c r="E37" t="str">
-        <v>$/unit</v>
-      </c>
-      <c r="F37" t="str">
-        <v>Ext $</v>
-      </c>
-      <c r="G37" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v/>
+        <v>Material #</v>
       </c>
       <c r="B38" t="str">
-        <v>Mojo Salmon</v>
+        <v>Variety</v>
       </c>
       <c r="C38" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D38">
-        <v>600</v>
-      </c>
-      <c r="E38">
-        <v>0.5243</v>
-      </c>
-      <c r="F38">
-        <v>314.57</v>
+        <v>Form</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Qty</v>
+      </c>
+      <c r="E38" t="str">
+        <v>$/unit</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Ext $</v>
       </c>
       <c r="G38" t="str">
-        <v/>
+        <v>Notes</v>
       </c>
     </row>
     <row r="39">
@@ -1150,19 +1150,19 @@
         <v/>
       </c>
       <c r="B39" t="str">
-        <v>Calliope Medium Pink Flame</v>
+        <v>Mojo Salmon</v>
       </c>
       <c r="C39" t="str">
         <v>CALL</v>
       </c>
       <c r="D39">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="E39">
-        <v>0.5983</v>
+        <v>0.5243</v>
       </c>
       <c r="F39">
-        <v>299.13</v>
+        <v>157.29</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -1173,19 +1173,19 @@
         <v/>
       </c>
       <c r="B40" t="str">
-        <v>Calliope Medium Hot Rose</v>
+        <v>Caldera Lavender Glow</v>
       </c>
       <c r="C40" t="str">
         <v>CALL</v>
       </c>
       <c r="D40">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="E40">
-        <v>0.5983</v>
+        <v>0.5243</v>
       </c>
       <c r="F40">
-        <v>299.13</v>
+        <v>157.29</v>
       </c>
       <c r="G40" t="str">
         <v/>
@@ -1196,19 +1196,19 @@
         <v/>
       </c>
       <c r="B41" t="str">
-        <v>Calliope Medium Dark Red DL</v>
+        <v>Caldera Hot Pink</v>
       </c>
       <c r="C41" t="str">
         <v>CALL</v>
       </c>
       <c r="D41">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="E41">
-        <v>0.5983</v>
+        <v>0.5243</v>
       </c>
       <c r="F41">
-        <v>598.27</v>
+        <v>157.29</v>
       </c>
       <c r="G41" t="str">
         <v/>
@@ -1219,128 +1219,128 @@
         <v/>
       </c>
       <c r="B42" t="str">
-        <v>ORDER TOTAL</v>
+        <v>Calliope Medium Pink Flame</v>
       </c>
       <c r="C42" t="str">
-        <v/>
+        <v>CALL</v>
       </c>
       <c r="D42">
-        <v>2600</v>
-      </c>
-      <c r="E42" t="str">
-        <v/>
+        <v>300</v>
+      </c>
+      <c r="E42">
+        <v>0.5983</v>
       </c>
       <c r="F42">
-        <v>1511.1</v>
+        <v>179.48</v>
       </c>
       <c r="G42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v/>
+      </c>
+      <c r="B43" t="str">
+        <v>Calliope Medium Hot Rose</v>
+      </c>
+      <c r="C43" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D43">
+        <v>300</v>
+      </c>
+      <c r="E43">
+        <v>0.5983</v>
+      </c>
+      <c r="F43">
+        <v>179.48</v>
+      </c>
+      <c r="G43" t="str">
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ORDER DRAFT-EHR-SYNG-SYNG-2711</v>
+        <v/>
       </c>
       <c r="B44" t="str">
-        <v>EHR → Syngenta — Syngenta Mexico</v>
+        <v>Calliope Medium Dark Red DL</v>
       </c>
       <c r="C44" t="str">
-        <v>Ship wk 11 (2027-03-15)</v>
-      </c>
-      <c r="D44" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D44">
+        <v>1200</v>
+      </c>
+      <c r="E44">
+        <v>0.5983</v>
+      </c>
+      <c r="F44">
+        <v>717.92</v>
+      </c>
+      <c r="G44" t="str">
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Material #</v>
+        <v/>
       </c>
       <c r="B45" t="str">
-        <v>Variety</v>
+        <v>ORDER TOTAL</v>
       </c>
       <c r="C45" t="str">
-        <v>Form</v>
-      </c>
-      <c r="D45" t="str">
-        <v>Qty</v>
+        <v/>
+      </c>
+      <c r="D45">
+        <v>2700</v>
       </c>
       <c r="E45" t="str">
-        <v>$/unit</v>
-      </c>
-      <c r="F45" t="str">
-        <v>Ext $</v>
+        <v/>
+      </c>
+      <c r="F45">
+        <v>1548.75</v>
       </c>
       <c r="G45" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v/>
-      </c>
-      <c r="B46" t="str">
-        <v>Mojo Salmon</v>
-      </c>
-      <c r="C46" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D46">
-        <v>500</v>
-      </c>
-      <c r="E46">
-        <v>0.5243</v>
-      </c>
-      <c r="F46">
-        <v>262.15</v>
-      </c>
-      <c r="G46" t="str">
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v/>
+        <v>ORDER DRAFT-EHR-SYNG-SYNG-2710</v>
       </c>
       <c r="B47" t="str">
-        <v>Calliope Medium Pink Flame</v>
+        <v>EHR → Syngenta — Syngenta Mexico</v>
       </c>
       <c r="C47" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D47">
-        <v>500</v>
-      </c>
-      <c r="E47">
-        <v>0.5983</v>
-      </c>
-      <c r="F47">
-        <v>299.13</v>
-      </c>
-      <c r="G47" t="str">
+        <v>Ship wk 10 (2027-03-08)</v>
+      </c>
+      <c r="D47" t="str">
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>Material #</v>
       </c>
       <c r="B48" t="str">
-        <v>Calliope Medium Hot Rose</v>
+        <v>Variety</v>
       </c>
       <c r="C48" t="str">
-        <v>CALL</v>
-      </c>
-      <c r="D48">
-        <v>500</v>
-      </c>
-      <c r="E48">
-        <v>0.5983</v>
-      </c>
-      <c r="F48">
-        <v>299.13</v>
+        <v>Form</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Qty</v>
+      </c>
+      <c r="E48" t="str">
+        <v>$/unit</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Ext $</v>
       </c>
       <c r="G48" t="str">
-        <v/>
+        <v>Notes</v>
       </c>
     </row>
     <row r="49">
@@ -1348,19 +1348,19 @@
         <v/>
       </c>
       <c r="B49" t="str">
-        <v>Calliope Medium Dark Red DL</v>
+        <v>Mojo Salmon</v>
       </c>
       <c r="C49" t="str">
         <v>CALL</v>
       </c>
       <c r="D49">
-        <v>1500</v>
+        <v>600</v>
       </c>
       <c r="E49">
-        <v>0.5983</v>
+        <v>0.5243</v>
       </c>
       <c r="F49">
-        <v>897.4</v>
+        <v>314.57</v>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -1371,21 +1371,44 @@
         <v/>
       </c>
       <c r="B50" t="str">
-        <v>ORDER TOTAL</v>
+        <v>Calliope Medium Pink Flame</v>
       </c>
       <c r="C50" t="str">
-        <v/>
+        <v>CALL</v>
       </c>
       <c r="D50">
-        <v>3000</v>
-      </c>
-      <c r="E50" t="str">
-        <v/>
+        <v>500</v>
+      </c>
+      <c r="E50">
+        <v>0.5983</v>
       </c>
       <c r="F50">
-        <v>1757.81</v>
+        <v>299.13</v>
       </c>
       <c r="G50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v/>
+      </c>
+      <c r="B51" t="str">
+        <v>Calliope Medium Hot Rose</v>
+      </c>
+      <c r="C51" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D51">
+        <v>500</v>
+      </c>
+      <c r="E51">
+        <v>0.5983</v>
+      </c>
+      <c r="F51">
+        <v>299.13</v>
+      </c>
+      <c r="G51" t="str">
         <v/>
       </c>
     </row>
@@ -1394,27 +1417,225 @@
         <v/>
       </c>
       <c r="B52" t="str">
-        <v>GRAND TOTAL — 6 orders</v>
+        <v>Calliope Medium Dark Red DL</v>
       </c>
       <c r="C52" t="str">
-        <v/>
+        <v>CALL</v>
       </c>
       <c r="D52">
-        <v>14600</v>
-      </c>
-      <c r="E52" t="str">
-        <v/>
+        <v>1000</v>
+      </c>
+      <c r="E52">
+        <v>0.5983</v>
       </c>
       <c r="F52">
-        <v>8484.68</v>
+        <v>598.27</v>
       </c>
       <c r="G52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v/>
+      </c>
+      <c r="B53" t="str">
+        <v>ORDER TOTAL</v>
+      </c>
+      <c r="C53" t="str">
+        <v/>
+      </c>
+      <c r="D53">
+        <v>2600</v>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53">
+        <v>1511.1</v>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>ORDER DRAFT-EHR-SYNG-SYNG-2711</v>
+      </c>
+      <c r="B55" t="str">
+        <v>EHR → Syngenta — Syngenta Mexico</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Ship wk 11 (2027-03-15)</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Material #</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Variety</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Form</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Qty</v>
+      </c>
+      <c r="E56" t="str">
+        <v>$/unit</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Ext $</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v/>
+      </c>
+      <c r="B57" t="str">
+        <v>Mojo Salmon</v>
+      </c>
+      <c r="C57" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D57">
+        <v>500</v>
+      </c>
+      <c r="E57">
+        <v>0.5243</v>
+      </c>
+      <c r="F57">
+        <v>262.15</v>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v/>
+      </c>
+      <c r="B58" t="str">
+        <v>Calliope Medium Pink Flame</v>
+      </c>
+      <c r="C58" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D58">
+        <v>500</v>
+      </c>
+      <c r="E58">
+        <v>0.5983</v>
+      </c>
+      <c r="F58">
+        <v>299.13</v>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v/>
+      </c>
+      <c r="B59" t="str">
+        <v>Calliope Medium Hot Rose</v>
+      </c>
+      <c r="C59" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D59">
+        <v>500</v>
+      </c>
+      <c r="E59">
+        <v>0.5983</v>
+      </c>
+      <c r="F59">
+        <v>299.13</v>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v/>
+      </c>
+      <c r="B60" t="str">
+        <v>Calliope Medium Dark Red DL</v>
+      </c>
+      <c r="C60" t="str">
+        <v>CALL</v>
+      </c>
+      <c r="D60">
+        <v>1500</v>
+      </c>
+      <c r="E60">
+        <v>0.5983</v>
+      </c>
+      <c r="F60">
+        <v>897.4</v>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v/>
+      </c>
+      <c r="B61" t="str">
+        <v>ORDER TOTAL</v>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61">
+        <v>3000</v>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61">
+        <v>1757.81</v>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v/>
+      </c>
+      <c r="B63" t="str">
+        <v>GRAND TOTAL — 7 orders</v>
+      </c>
+      <c r="C63" t="str">
+        <v/>
+      </c>
+      <c r="D63">
+        <v>18300</v>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+      <c r="F63">
+        <v>10249.65</v>
+      </c>
+      <c r="G63" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>